<commit_message>
UI tests with Jest and Testing Library for the stepper, upload and setup screens, plus CSV and XLSX success and failure fixtures
</commit_message>
<xml_diff>
--- a/apps/api/fixtures/sample_portfolio_bengaluru.xlsx
+++ b/apps/api/fixtures/sample_portfolio_bengaluru.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="36">
   <si>
     <t>store_name</t>
   </si>
@@ -37,7 +37,15 @@
     <t>longitude</t>
   </si>
   <si>
-    <t>FreshMart Koramangala</t>
+    <r>
+      <rPr>
+        <b/>
+      </rPr>
+      <t xml:space="preserve">FreshMart </t>
+    </r>
+    <r>
+      <t>Koramangala</t>
+    </r>
   </si>
   <si>
     <t>80 Feet Road, Koramangala 4th Block</t>
@@ -55,12 +63,6 @@
     <t>Supermarket</t>
   </si>
   <si>
-    <t>12.9352</t>
-  </si>
-  <si>
-    <t>77.6245</t>
-  </si>
-  <si>
     <t>MediPlus Pharmacy Indiranagar</t>
   </si>
   <si>
@@ -70,12 +72,6 @@
     <t>Pharmacy</t>
   </si>
   <si>
-    <t>12.9719</t>
-  </si>
-  <si>
-    <t>77.6412</t>
-  </si>
-  <si>
     <t>BigBasket Hyperstore Whitefield</t>
   </si>
   <si>
@@ -85,9 +81,6 @@
     <t>Hypermarket</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>Daily Needs Grocery HSR</t>
   </si>
   <si>
@@ -97,24 +90,12 @@
     <t>Grocery Store</t>
   </si>
   <si>
-    <t>12.9121</t>
-  </si>
-  <si>
-    <t>77.6446</t>
-  </si>
-  <si>
     <t>Apollo Pharmacy Jayanagar</t>
   </si>
   <si>
     <t>4th Block, Jayanagar</t>
   </si>
   <si>
-    <t>12.9250</t>
-  </si>
-  <si>
-    <t>77.5938</t>
-  </si>
-  <si>
     <t>More Supermarket JP Nagar</t>
   </si>
   <si>
@@ -127,12 +108,6 @@
     <t>Sampige Road, Malleswaram</t>
   </si>
   <si>
-    <t>13.0035</t>
-  </si>
-  <si>
-    <t>77.5709</t>
-  </si>
-  <si>
     <t>Corner Store Marathahalli</t>
   </si>
   <si>
@@ -142,22 +117,10 @@
     <t>Convenience Store</t>
   </si>
   <si>
-    <t>12.9569</t>
-  </si>
-  <si>
-    <t>77.7011</t>
-  </si>
-  <si>
     <t>Nilgiris Grocery BTM Layout</t>
   </si>
   <si>
     <t>29th Main Road, BTM Layout 2nd Stage</t>
-  </si>
-  <si>
-    <t>12.9166</t>
-  </si>
-  <si>
-    <t>77.6101</t>
   </si>
   <si>
     <t>Wellness Forever Pharmacy Rajajinagar</t>
@@ -588,45 +551,45 @@
       <c r="F2" t="s">
         <v>13</v>
       </c>
-      <c r="G2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H2" t="s">
-        <v>15</v>
+      <c r="G2">
+        <v>12.9352</v>
+      </c>
+      <c r="H2">
+        <v>77.6245</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" t="s">
         <v>16</v>
       </c>
-      <c r="B3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F3" t="s">
-        <v>18</v>
-      </c>
-      <c r="G3" t="s">
-        <v>19</v>
-      </c>
-      <c r="H3" t="s">
-        <v>20</v>
+      <c r="G3">
+        <v>12.9719</v>
+      </c>
+      <c r="H3">
+        <v>77.6412</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B4" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="C4" t="s">
         <v>10</v>
@@ -638,21 +601,15 @@
         <v>12</v>
       </c>
       <c r="F4" t="s">
-        <v>23</v>
-      </c>
-      <c r="G4" t="s">
-        <v>24</v>
-      </c>
-      <c r="H4" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B5" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C5" t="s">
         <v>10</v>
@@ -664,21 +621,21 @@
         <v>12</v>
       </c>
       <c r="F5" t="s">
-        <v>27</v>
-      </c>
-      <c r="G5" t="s">
-        <v>28</v>
-      </c>
-      <c r="H5" t="s">
-        <v>29</v>
+        <v>22</v>
+      </c>
+      <c r="G5">
+        <v>12.9121</v>
+      </c>
+      <c r="H5">
+        <v>77.6446</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="B6" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="C6" t="s">
         <v>10</v>
@@ -690,21 +647,21 @@
         <v>12</v>
       </c>
       <c r="F6" t="s">
-        <v>18</v>
-      </c>
-      <c r="G6" t="s">
-        <v>32</v>
-      </c>
-      <c r="H6" t="s">
-        <v>33</v>
+        <v>16</v>
+      </c>
+      <c r="G6">
+        <v>12.925</v>
+      </c>
+      <c r="H6">
+        <v>77.5938</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="B7" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="C7" t="s">
         <v>10</v>
@@ -718,19 +675,13 @@
       <c r="F7" t="s">
         <v>13</v>
       </c>
-      <c r="G7" t="s">
-        <v>24</v>
-      </c>
-      <c r="H7" t="s">
-        <v>24</v>
-      </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="B8" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="C8" t="s">
         <v>10</v>
@@ -742,21 +693,21 @@
         <v>12</v>
       </c>
       <c r="F8" t="s">
-        <v>23</v>
-      </c>
-      <c r="G8" t="s">
-        <v>38</v>
-      </c>
-      <c r="H8" t="s">
-        <v>39</v>
+        <v>19</v>
+      </c>
+      <c r="G8">
+        <v>13.0035</v>
+      </c>
+      <c r="H8">
+        <v>77.5709</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="B9" t="s">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="C9" t="s">
         <v>10</v>
@@ -768,21 +719,21 @@
         <v>12</v>
       </c>
       <c r="F9" t="s">
-        <v>42</v>
-      </c>
-      <c r="G9" t="s">
-        <v>43</v>
-      </c>
-      <c r="H9" t="s">
-        <v>44</v>
+        <v>31</v>
+      </c>
+      <c r="G9">
+        <v>12.9569</v>
+      </c>
+      <c r="H9">
+        <v>77.7011</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>45</v>
+        <v>32</v>
       </c>
       <c r="B10" t="s">
-        <v>46</v>
+        <v>33</v>
       </c>
       <c r="C10" t="s">
         <v>10</v>
@@ -794,21 +745,21 @@
         <v>12</v>
       </c>
       <c r="F10" t="s">
-        <v>27</v>
-      </c>
-      <c r="G10" t="s">
-        <v>47</v>
-      </c>
-      <c r="H10" t="s">
-        <v>48</v>
+        <v>22</v>
+      </c>
+      <c r="G10">
+        <v>12.9166</v>
+      </c>
+      <c r="H10">
+        <v>77.6101</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="B11" t="s">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="C11" t="s">
         <v>10</v>
@@ -820,13 +771,7 @@
         <v>12</v>
       </c>
       <c r="F11" t="s">
-        <v>18</v>
-      </c>
-      <c r="G11" t="s">
-        <v>24</v>
-      </c>
-      <c r="H11" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>